<commit_message>
Septiembre 2026 v2: incidencias revisadas el 07/10 y web con contraseña
- Albaranes v2: detalle de los tres tickets de Voldis reescaneados, ticket de Hielos del 29/08 y cargas de tanque de Mahou con importe estimado (4,00 EUR/l)
- Incidencias con ACCION, DEPARTAMENTO y RESULTADO: 32 pendientes, 16 cerradas
- Comparativa y control de PDF actualizados
- index.html: web de compras y precios con pantalla de contraseña (igual que la de Velázquez), datos nuevos y filtro por departamento

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012r9PcHpBkD5WrNbG83TmsE
</commit_message>
<xml_diff>
--- a/2026/3t/SEPTIEMBRE/ALBARANES/CONTROL PDF LA MINA CHAMARTIN SEPTIEMBRE 2026.xlsx
+++ b/2026/3t/SEPTIEMBRE/ALBARANES/CONTROL PDF LA MINA CHAMARTIN SEPTIEMBRE 2026.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DETALLE" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DETALLE'!$A$1:$L$326</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DETALLE'!$A$1:$L$332</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -536,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:I23"/>
+  <dimension ref="B2:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -597,7 +597,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>NO INCLUIDOS (revisar)</t>
+          <t>NO INCLUIDOS (no son albarán valorado)</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -619,16 +619,16 @@
         <v>70</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="G6" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I6" s="5" t="n">
         <v>0</v>
@@ -650,7 +650,7 @@
         <v>73</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="G7" s="5" t="n">
         <v>0</v>
@@ -675,16 +675,16 @@
         <v>30</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G8" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8" s="5" t="n">
         <v>0</v>
@@ -703,16 +703,16 @@
         <v>103</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="G9" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I9" s="5" t="n">
         <v>0</v>
@@ -762,7 +762,7 @@
         <v>33</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G11" s="5" t="n">
         <v>0</v>
@@ -775,112 +775,148 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>procesados/Scanned-image07-10-2026-105415.pdf (reescaneo de 3 tickets de Voldis)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>procesados/Scanned-image07-10-2026-105610.pdf (reescaneo de 3 tickets de Voldis)</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C12" s="6">
-        <f>SUM(C6:C11)</f>
+      <c r="C14" s="6">
+        <f>SUM(C6:C13)</f>
         <v/>
       </c>
-      <c r="D12" s="6">
-        <f>SUM(D6:D11)</f>
+      <c r="D14" s="6">
+        <f>SUM(D6:D13)</f>
         <v/>
       </c>
-      <c r="E12" s="6">
-        <f>SUM(E6:E11)</f>
+      <c r="E14" s="6">
+        <f>SUM(E6:E13)</f>
         <v/>
       </c>
-      <c r="F12" s="6">
-        <f>SUM(F6:F11)</f>
+      <c r="F14" s="6">
+        <f>SUM(F6:F13)</f>
         <v/>
       </c>
-      <c r="G12" s="6">
-        <f>SUM(G6:G11)</f>
+      <c r="G14" s="6">
+        <f>SUM(G6:G13)</f>
         <v/>
       </c>
-      <c r="H12" s="6">
-        <f>SUM(H6:H11)</f>
+      <c r="H14" s="6">
+        <f>SUM(H6:H13)</f>
         <v/>
       </c>
-      <c r="I12" s="6">
-        <f>SUM(I6:I11)</f>
+      <c r="I14" s="6">
+        <f>SUM(I6:I13)</f>
         <v/>
       </c>
     </row>
-    <row r="14" ht="52" customHeight="1">
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>✔ TODAS LAS PÁGINAS REVISADAS (301 páginas, 6 PDF). Todos los albaranes valorados de La Mina de Chamartín de estos PDF están en el Excel del mes. Lo que no se ha incluido es de otro cliente, de otro mes o viene sin valorar (ver hoja DETALLE e INCIDENCIAS). Ojo: en 2 páginas hay un albarán tapado por otro; están en el Excel solo por el importe que se ve.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="8" t="inlineStr">
+    <row r="16" ht="80" customHeight="1">
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>✔ TODAS LAS PÁGINAS REVISADAS (303 páginas, 8 PDF). Todos los albaranes valorados de La Mina de Chamartín de estos PDF están en el Excel del mes. Lo que no se ha incluido es de otro cliente o no es un albarán valorado: dos hojas de pedido, una factura y una muestra (ver hoja DETALLE e INCIDENCIAS). Ojo: en 2 páginas hay un albarán tapado por otro; están en el Excel solo por el importe que se ve. Los dos albaranes de tanque de Mahou van con importe estimado (4,00 €/l) hasta que llegue la factura. Los 2 PDF del 07/10 son reescaneos de tres tickets de Voldis que ya estaban contados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>CUADRE CON EL EXCEL DE ALBARANES</t>
         </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>Albaranes en el Excel del mes</t>
-        </is>
-      </c>
-      <c r="F17" s="10" t="n">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Líneas en TOTAL SEPTIEMBRE (albarán o tramo de IVA)</t>
-        </is>
-      </c>
-      <c r="F18" s="10" t="n">
-        <v>341</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Base total del Excel</t>
-        </is>
-      </c>
-      <c r="F19" s="11" t="n">
-        <v>65831.92</v>
+          <t>Albaranes en el Excel del mes</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="n">
+        <v>308</v>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Líneas que salen de estos PDF</t>
+          <t>Líneas en TOTAL SEPTIEMBRE (albarán o tramo de IVA)</t>
         </is>
       </c>
       <c r="F20" s="10" t="n">
-        <v>341</v>
+        <v>344</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Base de esas líneas</t>
+          <t>Base total del Excel</t>
         </is>
       </c>
       <c r="F21" s="11" t="n">
-        <v>65831.92</v>
+        <v>73621.92</v>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Líneas que NO salen de estos PDF</t>
+          <t>Líneas que salen de estos PDF</t>
         </is>
       </c>
       <c r="F22" s="10" t="n">
-        <v>0</v>
+        <v>344</v>
       </c>
     </row>
     <row r="23">
@@ -890,18 +926,38 @@
         </is>
       </c>
       <c r="F23" s="11" t="n">
+        <v>73621.92</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Líneas que NO salen de estos PDF</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Base de esas líneas</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="B18:E18"/>
     <mergeCell ref="B23:E23"/>
+    <mergeCell ref="B16:I16"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="B21:E21"/>
     <mergeCell ref="B3:I3"/>
-    <mergeCell ref="B14:I14"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B24:E24"/>
     <mergeCell ref="B19:E19"/>
     <mergeCell ref="B20:E20"/>
     <mergeCell ref="B22:E22"/>
@@ -917,7 +973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L326"/>
+  <dimension ref="A1:L332"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1081,12 +1137,12 @@
       </c>
       <c r="I3" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J3" s="9" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>65 (cerrada)</t>
         </is>
       </c>
       <c r="K3" s="14" t="inlineStr">
@@ -1288,7 +1344,7 @@
       </c>
       <c r="J7" s="9" t="inlineStr">
         <is>
-          <t>56, 65</t>
+          <t>56, 65 (cerrada)</t>
         </is>
       </c>
       <c r="K7" s="14" t="inlineStr">
@@ -1527,13 +1583,15 @@
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="H12" s="13" t="n"/>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="H12" s="13" t="n">
+        <v>3936</v>
+      </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>NO INCLUIDO (revisar)</t>
+          <t>OK CON INCIDENCIA</t>
         </is>
       </c>
       <c r="J12" s="9" t="inlineStr">
@@ -1548,7 +1606,7 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Albarán de entrega de cerveza de tanque: Mahou Clásica Duotank 1L, 1.000 L impreso (corregido a mano: 984). Sin precios.</t>
+          <t>Albarán de cerveza de tanque sin precios. Por indicación de la asesoría (07/10/2026) se valora al precio de la última carga facturada por Mahou (La Mina de Velázquez, septiembre): 3,90 €/l + 0,10 €/l de impuesto especial. A sustituir por el importe de la factura. 1.000 litros impresos, corregido a mano a 984 (se toman 984)</t>
         </is>
       </c>
     </row>
@@ -1871,12 +1929,12 @@
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J19" s="9" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>65 (cerrada)</t>
         </is>
       </c>
       <c r="K19" s="14" t="inlineStr">
@@ -2017,12 +2075,12 @@
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J22" s="9" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>65 (cerrada)</t>
         </is>
       </c>
       <c r="K22" s="14" t="inlineStr">
@@ -2765,12 +2823,12 @@
       </c>
       <c r="I37" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J37" s="9" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>67 (cerrada)</t>
         </is>
       </c>
       <c r="K37" s="14" t="inlineStr">
@@ -2909,12 +2967,12 @@
       <c r="H40" s="13" t="n"/>
       <c r="I40" s="9" t="inlineStr">
         <is>
-          <t>NO INCLUIDO (revisar)</t>
+          <t>NO INCLUIDO (revisado)</t>
         </is>
       </c>
       <c r="J40" s="9" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>61 (cerrada)</t>
         </is>
       </c>
       <c r="K40" s="14" t="inlineStr">
@@ -2967,12 +3025,12 @@
       </c>
       <c r="I41" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J41" s="9" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>62 (cerrada)</t>
         </is>
       </c>
       <c r="K41" s="14" t="inlineStr">
@@ -3071,12 +3129,12 @@
       </c>
       <c r="I43" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J43" s="9" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>62 (cerrada)</t>
         </is>
       </c>
       <c r="K43" s="14" t="inlineStr">
@@ -3558,7 +3616,7 @@
       </c>
       <c r="J53" s="9" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>46 (cerrada)</t>
         </is>
       </c>
       <c r="K53" s="14" t="inlineStr">
@@ -4919,12 +4977,12 @@
       </c>
       <c r="I81" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J81" s="9" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>62 (cerrada)</t>
         </is>
       </c>
       <c r="K81" s="14" t="inlineStr">
@@ -4977,12 +5035,12 @@
       </c>
       <c r="I82" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J82" s="9" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>62 (cerrada)</t>
         </is>
       </c>
       <c r="K82" s="14" t="inlineStr">
@@ -5081,12 +5139,12 @@
       </c>
       <c r="I84" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J84" s="9" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>65 (cerrada)</t>
         </is>
       </c>
       <c r="K84" s="14" t="inlineStr">
@@ -6073,12 +6131,12 @@
       </c>
       <c r="I105" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J105" s="9" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>62 (cerrada)</t>
         </is>
       </c>
       <c r="K105" s="14" t="inlineStr">
@@ -6131,12 +6189,12 @@
       </c>
       <c r="I106" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J106" s="9" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>67 (cerrada)</t>
         </is>
       </c>
       <c r="K106" s="14" t="inlineStr">
@@ -6873,12 +6931,12 @@
       <c r="H122" s="13" t="n"/>
       <c r="I122" s="9" t="inlineStr">
         <is>
-          <t>NO INCLUIDO (revisar)</t>
+          <t>NO INCLUIDO (revisado)</t>
         </is>
       </c>
       <c r="J122" s="9" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>58 (cerrada)</t>
         </is>
       </c>
       <c r="K122" s="14" t="inlineStr">
@@ -7763,12 +7821,12 @@
       </c>
       <c r="I140" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J140" s="9" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>67 (cerrada)</t>
         </is>
       </c>
       <c r="K140" s="14" t="inlineStr">
@@ -8287,12 +8345,12 @@
       </c>
       <c r="I151" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J151" s="9" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>62 (cerrada)</t>
         </is>
       </c>
       <c r="K151" s="14" t="inlineStr">
@@ -8559,18 +8617,20 @@
       </c>
       <c r="G156" s="9" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="H156" s="13" t="n"/>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="H156" s="13" t="n">
+        <v>50</v>
+      </c>
       <c r="I156" s="9" t="inlineStr">
         <is>
-          <t>NO INCLUIDO (revisar)</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J156" s="9" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>45 (cerrada)</t>
         </is>
       </c>
       <c r="K156" s="14" t="inlineStr">
@@ -8580,7 +8640,7 @@
       </c>
       <c r="L156" s="9" t="inlineStr">
         <is>
-          <t>Ticket del 29/08/2026 (agosto), a nombre de "La Mina Chamartín": 10 sacos hielo cocktelería = 50,00 €. Lleva escrito "EXCEL" rodeado. Es de agosto y llega con los de septiembre.</t>
+          <t>Ticket manuscrito sin nº ni IVA, del 29/08/2026, a nombre de "La Mina Chamartín". Lleva escrito "EXCEL". Llegó con los de septiembre y se incluye en septiembre por indicación de la asesoría (07/10/2026)</t>
         </is>
       </c>
     </row>
@@ -9259,12 +9319,12 @@
       </c>
       <c r="I169" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J169" s="9" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>50 (cerrada)</t>
         </is>
       </c>
       <c r="K169" s="14" t="inlineStr">
@@ -9274,7 +9334,7 @@
       </c>
       <c r="L169" s="9" t="inlineStr">
         <is>
-          <t>Copia casi en blanco; solo se leen las cantidades (4 berberecho, 2 chochas gda, 5 mejillones). Precios e importe puestos con los precios habituales del mes (22 / 50 / 2,70); fecha ilegible</t>
+          <t>Copia casi en blanco. Cantidades y precios confirmados por La Mina el 07/10/2026 (4 berberecho a 22, 2 chochas a 50, 5 mejillones a 2,70); fecha ilegible</t>
         </is>
       </c>
     </row>
@@ -9997,12 +10057,12 @@
       </c>
       <c r="I184" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J184" s="9" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>62 (cerrada)</t>
         </is>
       </c>
       <c r="K184" s="14" t="inlineStr">
@@ -10055,12 +10115,12 @@
       </c>
       <c r="I185" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J185" s="9" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>62 (cerrada)</t>
         </is>
       </c>
       <c r="K185" s="14" t="inlineStr">
@@ -10118,7 +10178,7 @@
       </c>
       <c r="J186" s="9" t="inlineStr">
         <is>
-          <t>51, 62</t>
+          <t>51, 62 (cerrada)</t>
         </is>
       </c>
       <c r="K186" s="14" t="inlineStr">
@@ -10171,12 +10231,12 @@
       </c>
       <c r="I187" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J187" s="9" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>62 (cerrada)</t>
         </is>
       </c>
       <c r="K187" s="14" t="inlineStr">
@@ -10229,12 +10289,12 @@
       </c>
       <c r="I188" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J188" s="9" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>62 (cerrada)</t>
         </is>
       </c>
       <c r="K188" s="14" t="inlineStr">
@@ -10287,12 +10347,12 @@
       </c>
       <c r="I189" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J189" s="9" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>62 (cerrada)</t>
         </is>
       </c>
       <c r="K189" s="14" t="inlineStr">
@@ -10345,12 +10405,12 @@
       </c>
       <c r="I190" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J190" s="9" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>60 (cerrada)</t>
         </is>
       </c>
       <c r="K190" s="14" t="inlineStr">
@@ -10395,13 +10455,15 @@
       </c>
       <c r="G191" s="9" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="H191" s="13" t="n"/>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="H191" s="13" t="n">
+        <v>3804</v>
+      </c>
       <c r="I191" s="9" t="inlineStr">
         <is>
-          <t>NO INCLUIDO (revisar)</t>
+          <t>OK CON INCIDENCIA</t>
         </is>
       </c>
       <c r="J191" s="9" t="inlineStr">
@@ -10416,7 +10478,7 @@
       </c>
       <c r="L191" s="9" t="inlineStr">
         <is>
-          <t>Albarán de cerveza de tanque: 951 litros. Sin precios.</t>
+          <t>Albarán de cerveza de tanque sin precios. Por indicación de la asesoría (07/10/2026) se valora al precio de la última carga facturada por Mahou (La Mina de Velázquez, septiembre): 3,90 €/l + 0,10 €/l de impuesto especial. A sustituir por el importe de la factura. 951 litros</t>
         </is>
       </c>
     </row>
@@ -10459,12 +10521,12 @@
       </c>
       <c r="I192" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J192" s="9" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>62 (cerrada)</t>
         </is>
       </c>
       <c r="K192" s="14" t="inlineStr">
@@ -10517,12 +10579,12 @@
       </c>
       <c r="I193" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J193" s="9" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>62 (cerrada)</t>
         </is>
       </c>
       <c r="K193" s="14" t="inlineStr">
@@ -10575,12 +10637,12 @@
       </c>
       <c r="I194" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J194" s="9" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>62 (cerrada)</t>
         </is>
       </c>
       <c r="K194" s="14" t="inlineStr">
@@ -10679,12 +10741,12 @@
       </c>
       <c r="I196" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J196" s="9" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>59 (cerrada)</t>
         </is>
       </c>
       <c r="K196" s="14" t="inlineStr">
@@ -10733,12 +10795,12 @@
       </c>
       <c r="I197" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J197" s="9" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>59 (cerrada)</t>
         </is>
       </c>
       <c r="K197" s="14" t="inlineStr">
@@ -10791,12 +10853,12 @@
       </c>
       <c r="I198" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J198" s="9" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>53 (cerrada)</t>
         </is>
       </c>
       <c r="K198" s="14" t="inlineStr">
@@ -12253,12 +12315,12 @@
       </c>
       <c r="I229" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J229" s="9" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>53 (cerrada)</t>
         </is>
       </c>
       <c r="K229" s="14" t="inlineStr">
@@ -12403,12 +12465,12 @@
       </c>
       <c r="I232" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J232" s="9" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>53 (cerrada)</t>
         </is>
       </c>
       <c r="K232" s="14" t="inlineStr">
@@ -13105,12 +13167,12 @@
       </c>
       <c r="I247" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J247" s="9" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>53 (cerrada)</t>
         </is>
       </c>
       <c r="K247" s="14" t="inlineStr">
@@ -14003,12 +14065,12 @@
       </c>
       <c r="I266" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J266" s="9" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>59 (cerrada)</t>
         </is>
       </c>
       <c r="K266" s="14" t="inlineStr">
@@ -14153,12 +14215,12 @@
       </c>
       <c r="I269" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J269" s="9" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>59 (cerrada)</t>
         </is>
       </c>
       <c r="K269" s="14" t="inlineStr">
@@ -14533,12 +14595,12 @@
       </c>
       <c r="I277" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J277" s="9" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>67 (cerrada)</t>
         </is>
       </c>
       <c r="K277" s="14" t="inlineStr">
@@ -14656,7 +14718,7 @@
       </c>
       <c r="L279" s="9" t="inlineStr">
         <is>
-          <t>Albarán manuscrito escaneado debajo del de Peñalastallas 12377; solo se ve el pie: una línea a 35 = 38,50, subtotal 833,30 y total 916,6x. No se ven proveedor, fecha ni productos. Por el formato y los precios es de Pescarum y falta justo el del 05/09</t>
+          <t>Albarán manuscrito escaneado debajo del de Peñalastallas 12377; solo se ve el pie: una línea a 35 = 38,50, subtotal 833,30 y total 916,6x. No se ven proveedor, fecha ni productos. Por el formato y los precios es de Pescarum y falta justo el del 05/09. No es el del 04/09 (ese está entero en la página siguiente, con base 831,05)</t>
         </is>
       </c>
     </row>
@@ -14699,22 +14761,22 @@
       </c>
       <c r="I280" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J280" s="9" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>53 (cerrada), 68 (cerrada)</t>
         </is>
       </c>
       <c r="K280" s="14" t="inlineStr">
         <is>
-          <t>Lectura dudosa</t>
+          <t>Lectura dudosa; Total mal sumado</t>
         </is>
       </c>
       <c r="L280" s="9" t="inlineStr">
         <is>
-          <t>Pulpo: la cantidad parece 9,96 pero el importe (274,50) corresponde a 9,00 kg; se toma 9,00</t>
+          <t>Pulpo: la cantidad parece 9,96 pero el importe (274,50) corresponde a 9,00 kg; se toma 9,00. el albarán pone base 831,05 + IVA 83,10 y total 914,55 (la suma es 914,15)</t>
         </is>
       </c>
     </row>
@@ -16662,7 +16724,7 @@
       </c>
       <c r="L318" s="9" t="inlineStr">
         <is>
-          <t>Ticket térmico tenue. Bases del desglose de IVA (251,41 al 10% y 380,47 al 21%) cuadran con el total; el detalle leído suma 0,09 € menos al 10%. Los envases de Solan (200 botellas y 10 cajas) vienen cargados</t>
+          <t>Ticket térmico tenue. Bases del desglose de IVA (251,41 al 10% y 380,47 al 21%) cuadran con el total; Los envases de Solan (200 botellas y 10 cajas) vienen cargados; las cajas son 33,09 € (3,31 €/caja, como en el ticket del 25/09)</t>
         </is>
       </c>
     </row>
@@ -16682,7 +16744,7 @@
       </c>
       <c r="D319" s="12" t="inlineStr">
         <is>
-          <t>AP26-0326?? (25/09)</t>
+          <t>AP26-032600</t>
         </is>
       </c>
       <c r="E319" s="9" t="inlineStr">
@@ -16705,12 +16767,12 @@
       </c>
       <c r="I319" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J319" s="9" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>40 (cerrada)</t>
         </is>
       </c>
       <c r="K319" s="14" t="inlineStr">
@@ -16720,7 +16782,7 @@
       </c>
       <c r="L319" s="9" t="inlineStr">
         <is>
-          <t>Ticket térmico tapado por una tira a lo largo; solo se leen bases (144,78 al 10% y 864,27 al 21%) y total. 21 artículos, con muchos envases</t>
+          <t>Reescaneado el 07/10/2026 (Scanned-image07-10-2026-105415 y 105610): se lee todo el detalle (21 artículos). Devuelven envases de Solan (-140 botellas, -7 cajas), Pepsi/Kas y Schweppes; cargan envases de Mahou y una tanqueta. El cargo logístico (3,50 €) queda bajo la tira: es la diferencia con la base al 21%</t>
         </is>
       </c>
     </row>
@@ -16809,12 +16871,12 @@
       </c>
       <c r="I321" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J321" s="9" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>40 (cerrada)</t>
         </is>
       </c>
       <c r="K321" s="14" t="inlineStr">
@@ -16824,7 +16886,7 @@
       </c>
       <c r="L321" s="9" t="inlineStr">
         <is>
-          <t>Los importes de línea quedan tapados por otro ticket; se leen bases (164,26 al 10% y 1.085,51 al 21%) y total (14 artículos). Lleva escrito "EXCEL AGORA"</t>
+          <t>Reescaneado el 07/10/2026 (Scanned-image07-10-2026-105415 y 105610): se lee todo el detalle (14 artículos). Lleva escrito "EXCEL AGORA". El cargo logístico (2,50 €) no se lee en el ticket: es la diferencia entre las líneas y la base al 21%</t>
         </is>
       </c>
     </row>
@@ -16948,7 +17010,7 @@
       </c>
       <c r="D324" s="12" t="inlineStr">
         <is>
-          <t>AP26-03159? (18/09)</t>
+          <t>AP26-031592</t>
         </is>
       </c>
       <c r="E324" s="9" t="inlineStr">
@@ -16971,12 +17033,12 @@
       </c>
       <c r="I324" s="9" t="inlineStr">
         <is>
-          <t>OK CON INCIDENCIA</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="J324" s="9" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>40 (cerrada)</t>
         </is>
       </c>
       <c r="K324" s="14" t="inlineStr">
@@ -16986,7 +17048,7 @@
       </c>
       <c r="L324" s="9" t="inlineStr">
         <is>
-          <t>Los importes de línea quedan fuera del borde del escaneo; se leen bases (194,17 al 10% y 924,39 al 21%) y total (12 artículos)</t>
+          <t>Reescaneado el 07/10/2026 (Scanned-image07-10-2026-105415 y 105610): se lee todo el detalle (12 artículos). El zumo de tomate va al 10%</t>
         </is>
       </c>
     </row>
@@ -17094,9 +17156,321 @@
         </is>
       </c>
     </row>
+    <row r="327" ht="15" customHeight="1">
+      <c r="A327" s="9" t="inlineStr">
+        <is>
+          <t>Scanned-image07-10-2026-105415.pdf</t>
+        </is>
+      </c>
+      <c r="B327" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C327" s="9" t="inlineStr">
+        <is>
+          <t>VOLDIS</t>
+        </is>
+      </c>
+      <c r="D327" s="12" t="inlineStr">
+        <is>
+          <t>AP26-031592</t>
+        </is>
+      </c>
+      <c r="E327" s="9" t="inlineStr">
+        <is>
+          <t>18/09</t>
+        </is>
+      </c>
+      <c r="F327" s="9" t="inlineStr">
+        <is>
+          <t>LA MINA DE CHAMARTÍN</t>
+        </is>
+      </c>
+      <c r="G327" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="H327" s="13" t="n"/>
+      <c r="I327" s="9" t="inlineStr">
+        <is>
+          <t>OK (reescaneo)</t>
+        </is>
+      </c>
+      <c r="J327" s="9" t="inlineStr">
+        <is>
+          <t>40 (cerrada)</t>
+        </is>
+      </c>
+      <c r="K327" s="14" t="n"/>
+      <c r="L327" s="9" t="inlineStr">
+        <is>
+          <t>Reescaneo del 07/10/2026 del ticket AP26-031592: ya contado en Scanned-image05-10-2026-124247.pdf, página 10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="328" ht="15" customHeight="1">
+      <c r="A328" s="9" t="inlineStr">
+        <is>
+          <t>Scanned-image07-10-2026-105415.pdf</t>
+        </is>
+      </c>
+      <c r="B328" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C328" s="9" t="inlineStr">
+        <is>
+          <t>VOLDIS</t>
+        </is>
+      </c>
+      <c r="D328" s="12" t="inlineStr">
+        <is>
+          <t>AP26-030095</t>
+        </is>
+      </c>
+      <c r="E328" s="9" t="inlineStr">
+        <is>
+          <t>08/09</t>
+        </is>
+      </c>
+      <c r="F328" s="9" t="inlineStr">
+        <is>
+          <t>LA MINA DE CHAMARTÍN</t>
+        </is>
+      </c>
+      <c r="G328" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="H328" s="13" t="n"/>
+      <c r="I328" s="9" t="inlineStr">
+        <is>
+          <t>OK (reescaneo)</t>
+        </is>
+      </c>
+      <c r="J328" s="9" t="inlineStr">
+        <is>
+          <t>40 (cerrada)</t>
+        </is>
+      </c>
+      <c r="K328" s="14" t="n"/>
+      <c r="L328" s="9" t="inlineStr">
+        <is>
+          <t>Reescaneo del 07/10/2026 del ticket AP26-030095: ya contado en Scanned-image05-10-2026-124247.pdf, página 10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="329" ht="15" customHeight="1">
+      <c r="A329" s="9" t="inlineStr">
+        <is>
+          <t>Scanned-image07-10-2026-105415.pdf</t>
+        </is>
+      </c>
+      <c r="B329" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C329" s="9" t="inlineStr">
+        <is>
+          <t>VOLDIS</t>
+        </is>
+      </c>
+      <c r="D329" s="12" t="inlineStr">
+        <is>
+          <t>AP26-032600</t>
+        </is>
+      </c>
+      <c r="E329" s="9" t="inlineStr">
+        <is>
+          <t>25/09</t>
+        </is>
+      </c>
+      <c r="F329" s="9" t="inlineStr">
+        <is>
+          <t>LA MINA DE CHAMARTÍN</t>
+        </is>
+      </c>
+      <c r="G329" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="H329" s="13" t="n"/>
+      <c r="I329" s="9" t="inlineStr">
+        <is>
+          <t>OK (reescaneo)</t>
+        </is>
+      </c>
+      <c r="J329" s="9" t="inlineStr">
+        <is>
+          <t>40 (cerrada)</t>
+        </is>
+      </c>
+      <c r="K329" s="14" t="n"/>
+      <c r="L329" s="9" t="inlineStr">
+        <is>
+          <t>Reescaneo del 07/10/2026 del ticket AP26-032600: ya contado en Scanned-image05-10-2026-124247.pdf, página 9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="330" ht="15" customHeight="1">
+      <c r="A330" s="9" t="inlineStr">
+        <is>
+          <t>Scanned-image07-10-2026-105610.pdf</t>
+        </is>
+      </c>
+      <c r="B330" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C330" s="9" t="inlineStr">
+        <is>
+          <t>VOLDIS</t>
+        </is>
+      </c>
+      <c r="D330" s="12" t="inlineStr">
+        <is>
+          <t>AP26-031592</t>
+        </is>
+      </c>
+      <c r="E330" s="9" t="inlineStr">
+        <is>
+          <t>18/09</t>
+        </is>
+      </c>
+      <c r="F330" s="9" t="inlineStr">
+        <is>
+          <t>LA MINA DE CHAMARTÍN</t>
+        </is>
+      </c>
+      <c r="G330" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="H330" s="13" t="n"/>
+      <c r="I330" s="9" t="inlineStr">
+        <is>
+          <t>OK (reescaneo)</t>
+        </is>
+      </c>
+      <c r="J330" s="9" t="inlineStr">
+        <is>
+          <t>40 (cerrada)</t>
+        </is>
+      </c>
+      <c r="K330" s="14" t="n"/>
+      <c r="L330" s="9" t="inlineStr">
+        <is>
+          <t>Reescaneo del 07/10/2026 del ticket AP26-031592: ya contado en Scanned-image05-10-2026-124247.pdf, página 10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="331" ht="15" customHeight="1">
+      <c r="A331" s="9" t="inlineStr">
+        <is>
+          <t>Scanned-image07-10-2026-105610.pdf</t>
+        </is>
+      </c>
+      <c r="B331" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C331" s="9" t="inlineStr">
+        <is>
+          <t>VOLDIS</t>
+        </is>
+      </c>
+      <c r="D331" s="12" t="inlineStr">
+        <is>
+          <t>AP26-030095</t>
+        </is>
+      </c>
+      <c r="E331" s="9" t="inlineStr">
+        <is>
+          <t>08/09</t>
+        </is>
+      </c>
+      <c r="F331" s="9" t="inlineStr">
+        <is>
+          <t>LA MINA DE CHAMARTÍN</t>
+        </is>
+      </c>
+      <c r="G331" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="H331" s="13" t="n"/>
+      <c r="I331" s="9" t="inlineStr">
+        <is>
+          <t>OK (reescaneo)</t>
+        </is>
+      </c>
+      <c r="J331" s="9" t="inlineStr">
+        <is>
+          <t>40 (cerrada)</t>
+        </is>
+      </c>
+      <c r="K331" s="14" t="n"/>
+      <c r="L331" s="9" t="inlineStr">
+        <is>
+          <t>Reescaneo del 07/10/2026 del ticket AP26-030095: ya contado en Scanned-image05-10-2026-124247.pdf, página 10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="332" ht="15" customHeight="1">
+      <c r="A332" s="9" t="inlineStr">
+        <is>
+          <t>Scanned-image07-10-2026-105610.pdf</t>
+        </is>
+      </c>
+      <c r="B332" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C332" s="9" t="inlineStr">
+        <is>
+          <t>VOLDIS</t>
+        </is>
+      </c>
+      <c r="D332" s="12" t="inlineStr">
+        <is>
+          <t>AP26-032600</t>
+        </is>
+      </c>
+      <c r="E332" s="9" t="inlineStr">
+        <is>
+          <t>25/09</t>
+        </is>
+      </c>
+      <c r="F332" s="9" t="inlineStr">
+        <is>
+          <t>LA MINA DE CHAMARTÍN</t>
+        </is>
+      </c>
+      <c r="G332" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="H332" s="13" t="n"/>
+      <c r="I332" s="9" t="inlineStr">
+        <is>
+          <t>OK (reescaneo)</t>
+        </is>
+      </c>
+      <c r="J332" s="9" t="inlineStr">
+        <is>
+          <t>40 (cerrada)</t>
+        </is>
+      </c>
+      <c r="K332" s="14" t="n"/>
+      <c r="L332" s="9" t="inlineStr">
+        <is>
+          <t>Reescaneo del 07/10/2026 del ticket AP26-032600: ya contado en Scanned-image05-10-2026-124247.pdf, página 9.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L326"/>
-  <conditionalFormatting sqref="I2:I326">
+  <autoFilter ref="A1:L332"/>
+  <conditionalFormatting sqref="I2:I332">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK CON INCIDENCIA"</formula>
     </cfRule>

</xml_diff>